<commit_message>
Made cleaning pipeline account for the new 2024 data addition
</commit_message>
<xml_diff>
--- a/data_raw/data_raw_2024_sheets/LTER1_BR_P02_2024.xlsx
+++ b/data_raw/data_raw_2024_sheets/LTER1_BR_P02_2024.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/HLenihan 1/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryananderson/Reference/Bren/Coral Demography/data_raw/data_raw_2024_sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0BA2DEE-642D-B34A-9860-54C6E5842F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25CF06D-B90C-5D46-BAFE-566F8EF6FAB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6100" yWindow="1360" windowWidth="28900" windowHeight="22640" xr2:uid="{A2BB357F-CBBF-3E49-8FFC-BADB8B2820A4}"/>
+    <workbookView xWindow="1020" yWindow="560" windowWidth="28900" windowHeight="18780" xr2:uid="{A2BB357F-CBBF-3E49-8FFC-BADB8B2820A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$M$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$M$47</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="31">
   <si>
     <t>LTER1</t>
   </si>
@@ -194,7 +194,114 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="19">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF49900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF159FEC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF17A43F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFB0006"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFA1BCD6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFB07EDD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <sz val="11"/>
@@ -222,131 +329,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF49900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Calibri"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFB07EDD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFA1BCD6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFB0006"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF17A43F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF159FEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFA500"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFD4A6FF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -360,7 +343,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFD4A6FF"/>
+          <bgColor rgb="FFF49900"/>
         </patternFill>
       </fill>
     </dxf>
@@ -368,13 +351,6 @@
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF49900"/>
         </patternFill>
       </fill>
     </dxf>
@@ -732,7 +708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46ECC2C4-65F1-D042-8666-62EE02F3C86B}">
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2003,13 +1979,13 @@
         <v>5</v>
       </c>
       <c r="I38">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J38">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K38">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L38" t="s">
         <v>29</v>
@@ -2029,22 +2005,22 @@
         <v>8</v>
       </c>
       <c r="E39" s="4">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="F39">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="G39">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="I39">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J39">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K39">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L39" t="s">
         <v>29</v>
@@ -2064,13 +2040,13 @@
         <v>8</v>
       </c>
       <c r="E40" s="4">
-        <v>1.3</v>
+        <v>1.45</v>
       </c>
       <c r="F40">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="G40">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I40">
         <v>0.5</v>
@@ -2099,22 +2075,22 @@
         <v>8</v>
       </c>
       <c r="E41" s="4">
-        <v>1.45</v>
+        <v>1.89</v>
       </c>
       <c r="F41">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="G41">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="I41">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J41">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K41">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L41" t="s">
         <v>29</v>
@@ -2131,25 +2107,25 @@
         <v>7</v>
       </c>
       <c r="D42" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E42" s="4">
-        <v>1.89</v>
+        <v>2.5</v>
       </c>
       <c r="F42">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="G42">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="I42">
-        <v>1</v>
+        <v>3.8</v>
       </c>
       <c r="J42">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L42" t="s">
         <v>29</v>
@@ -2166,25 +2142,25 @@
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E43" s="4">
-        <v>2.5</v>
+        <v>2.73</v>
       </c>
       <c r="F43">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="G43">
         <v>80</v>
       </c>
       <c r="I43">
-        <v>3.8</v>
+        <v>2.5</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="K43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L43" t="s">
         <v>29</v>
@@ -2204,10 +2180,10 @@
         <v>8</v>
       </c>
       <c r="E44" s="4">
-        <v>2.73</v>
+        <v>2.69</v>
       </c>
       <c r="F44">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="G44">
         <v>80</v>
@@ -2239,19 +2215,19 @@
         <v>8</v>
       </c>
       <c r="E45" s="4">
-        <v>2.69</v>
+        <v>2.89</v>
       </c>
       <c r="F45">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="G45">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="I45">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="J45">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="K45">
         <v>1</v>
@@ -2274,13 +2250,13 @@
         <v>8</v>
       </c>
       <c r="E46" s="4">
-        <v>2.89</v>
+        <v>2.9</v>
       </c>
       <c r="F46">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="G46">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I46">
         <v>1</v>
@@ -2312,22 +2288,22 @@
         <v>2.9</v>
       </c>
       <c r="F47">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="G47">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="I47">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J47">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K47">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L47" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
@@ -2344,25 +2320,25 @@
         <v>8</v>
       </c>
       <c r="E48" s="4">
-        <v>2.9</v>
+        <v>7.05</v>
       </c>
       <c r="F48">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="G48">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="I48">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J48">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K48">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L48" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
@@ -2379,19 +2355,19 @@
         <v>8</v>
       </c>
       <c r="E49" s="4">
-        <v>7.05</v>
+        <v>2.89</v>
       </c>
       <c r="F49">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="G49">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="I49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K49">
         <v>2</v>
@@ -2400,117 +2376,74 @@
         <v>29</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" t="s">
-        <v>1</v>
-      </c>
-      <c r="C50" t="s">
-        <v>7</v>
-      </c>
-      <c r="D50" t="s">
-        <v>8</v>
-      </c>
-      <c r="E50" s="4">
-        <v>2.89</v>
-      </c>
-      <c r="F50">
-        <v>10</v>
-      </c>
-      <c r="G50">
-        <v>40</v>
-      </c>
-      <c r="I50">
-        <v>1</v>
-      </c>
-      <c r="J50">
-        <v>1</v>
-      </c>
-      <c r="K50">
-        <v>2</v>
-      </c>
-      <c r="L50" t="s">
-        <v>29</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A38:D49 D50">
-    <cfRule type="expression" dxfId="20" priority="3">
-      <formula>A38="UK"</formula>
+  <conditionalFormatting sqref="A38:D49 I31:K49 F38:G49">
+    <cfRule type="expression" dxfId="18" priority="1">
+      <formula>A31="UK"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="4">
-      <formula>A38="Na"</formula>
+    <cfRule type="expression" dxfId="17" priority="2">
+      <formula>A31="Na"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:H2">
-    <cfRule type="containsText" dxfId="18" priority="35" operator="containsText" text="Missing data">
+    <cfRule type="beginsWith" dxfId="16" priority="34" operator="beginsWith" text="FI">
+      <formula>LEFT(A2,LEN("FI"))="FI"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="35" operator="containsText" text="Missing data">
       <formula>NOT(ISERROR(SEARCH("Missing data",A2)))</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="17" priority="34" operator="beginsWith" text="FI">
-      <formula>LEFT(A2,LEN("FI"))="FI"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:M2">
-    <cfRule type="beginsWith" dxfId="16" priority="33" operator="beginsWith" text="FU">
+    <cfRule type="beginsWith" dxfId="14" priority="27" operator="beginsWith" text="UK">
+      <formula>LEFT(A2,LEN("UK"))="UK"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="13" priority="33" operator="beginsWith" text="FU">
       <formula>LEFT(A2,LEN("FU"))="FU"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="15" priority="27" operator="beginsWith" text="UK">
-      <formula>LEFT(A2,LEN("UK"))="UK"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3 A3:G23 I4:K4 I6:K6 I8:K8 H8:H9 H13 I14:K17 H15:H19 I19:K20 A24:H25 A26:G29 I27:K27 A30:K30 A31:G32 A33:H34 A35:G37">
+    <cfRule type="expression" dxfId="12" priority="36">
+      <formula>A3="UK"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3 A3:G23 I4:K4 I6:K6 I8:K8 H8:H9 H13 I14:K17 H15:H19 I19:K20 A24:H25 A26:G29 I27:K27 A30:K30 A31:G32 A33:H34 A35:G37 F38:G50 I31:K50">
-    <cfRule type="expression" dxfId="14" priority="37">
+    <cfRule type="expression" dxfId="11" priority="37">
       <formula>A3="Na"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="36">
-      <formula>A3="UK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3 H8:H9 H13 I15:K17 H15:H19 I19:K20 H24:H25 H30:K30 H33:H34">
-    <cfRule type="expression" dxfId="12" priority="43">
-      <formula>H3="Recruitment"</formula>
+    <cfRule type="containsText" dxfId="10" priority="38" operator="containsText" text=",">
+      <formula>NOT(ISERROR(SEARCH(",", H3)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="42">
+    <cfRule type="beginsWith" dxfId="9" priority="39" operator="beginsWith" text="Fusion">
+      <formula>LEFT(H3,LEN("Fusion"))="Fusion"</formula>
+    </cfRule>
+    <cfRule type="beginsWith" dxfId="8" priority="40" operator="beginsWith" text="Fission">
+      <formula>LEFT(H3,LEN("Fission"))="Fission"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="41">
+      <formula>H3="Death"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="42">
       <formula>H3="Growth"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="41">
-      <formula>H3="Death"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="9" priority="40" operator="beginsWith" text="Fission">
-      <formula>LEFT(H3,LEN("Fission"))="Fission"</formula>
-    </cfRule>
-    <cfRule type="beginsWith" dxfId="8" priority="39" operator="beginsWith" text="Fusion">
-      <formula>LEFT(H3,LEN("Fusion"))="Fusion"</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="38" operator="containsText" text=",">
-      <formula>NOT(ISERROR(SEARCH(",", H3)))</formula>
+    <cfRule type="expression" dxfId="5" priority="43">
+      <formula>H3="Recruitment"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="beginsWith" dxfId="6" priority="28" operator="beginsWith" text="FI">
+    <cfRule type="beginsWith" dxfId="4" priority="28" operator="beginsWith" text="FI">
       <formula>LEFT(I2,LEN("FI"))="FI"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="32" operator="containsText" text="D">
-      <formula>NOT(ISERROR(SEARCH("D",I2)))</formula>
+    <cfRule type="containsText" dxfId="3" priority="29" operator="containsText" text="Missing data">
+      <formula>NOT(ISERROR(SEARCH("Missing data",I2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="31" operator="containsText" text="NA">
+    <cfRule type="beginsWith" dxfId="2" priority="30" operator="beginsWith" text="R">
+      <formula>LEFT(I2,LEN("R"))="R"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="31" operator="containsText" text="NA">
       <formula>NOT(ISERROR(SEARCH("NA",I2)))</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="3" priority="30" operator="beginsWith" text="R">
-      <formula>LEFT(I2,LEN("R"))="R"</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="29" operator="containsText" text="Missing data">
-      <formula>NOT(ISERROR(SEARCH("Missing data",I2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A50:C50">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>A50="UK"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>A50="Na"</formula>
+    <cfRule type="containsText" dxfId="0" priority="32" operator="containsText" text="D">
+      <formula>NOT(ISERROR(SEARCH("D",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions gridLines="1"/>

</xml_diff>